<commit_message>
feat(monitoring): use real data for Excel report, split by product
Replace hardcoded export data with real timeline + product lookups:

- Hoist useStatusTimelineByIdHook and useProductHook into page
- buildRequestBodies groups RUNNING segments by productPartNo
- DANDORI segments shared across all product sections
- Customer/rpm from ProductData, operators from distinct userName
- Input header field = product RPM
- Date header = selectedDate (matches activity chart)
- Multi-sheet Excel: one sheet per product via fillTemplateMulti
- ExportPreview renders stacked sections with product separators
- API route accepts FillTemplateData[] (backward compatible)
</commit_message>
<xml_diff>
--- a/src/lib/template/excel-template.xlsx
+++ b/src/lib/template/excel-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\TOHO(Fajar)\KCF\MC Monitoring System\kcf-mc-monitoring\src\lib\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F3AE000-8F32-4628-AF2D-8874D6ED6F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103A4BE1-FA48-4A7A-9E2C-0AD2E0133893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A44CC11C-A6F5-42DE-B984-7CB6A06CB0CA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
     <t>Part Name</t>
   </si>
@@ -155,16 +155,22 @@
     <t>{{Result}}</t>
   </si>
   <si>
-    <t>( Produksi / Jam ({{Input}})  X  Lama Produksi )</t>
-  </si>
-  <si>
     <t>{{TotalCounterProduct}}</t>
   </si>
   <si>
     <t>%</t>
   </si>
   <si>
-    <t>Part NO</t>
+    <t>( Produksi / Jam ({{Rpm}})  X  Lama Produksi )</t>
+  </si>
+  <si>
+    <t>Part No</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>{{Customer}}</t>
   </si>
 </sst>
 </file>
@@ -237,7 +243,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -392,11 +398,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -435,6 +452,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -462,6 +491,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -471,116 +512,107 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,28 +971,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
       <c r="H4" s="5" t="s">
         <v>20</v>
       </c>
@@ -968,174 +1000,178 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="27" t="s">
+    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="66" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="61" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" s="62"/>
+      <c r="G6" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="H6" s="46"/>
+      <c r="I6" s="47"/>
+      <c r="J6" s="34" t="s">
+        <v>4</v>
+      </c>
+      <c r="K6" s="34"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="N6" s="34"/>
+    </row>
+    <row r="7" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="58"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="50"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
+      <c r="L7" s="55"/>
+      <c r="M7" s="55"/>
+      <c r="N7" s="55"/>
+    </row>
+    <row r="8" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="56" t="s">
+      <c r="C8" s="15"/>
+      <c r="D8" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="52" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="51"/>
-      <c r="G6" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="38"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="31" t="s">
-        <v>4</v>
-      </c>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31" t="s">
-        <v>5</v>
-      </c>
-      <c r="N6" s="31"/>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="56"/>
-      <c r="E7" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="47"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
-      <c r="M7" s="49"/>
-      <c r="N7" s="49"/>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
-      <c r="M8" s="49"/>
-      <c r="N8" s="49"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="27" t="s">
+      <c r="E8" s="64"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="50"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="55"/>
+    </row>
+    <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="67"/>
+      <c r="E9" s="61" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" s="62"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="55"/>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="M9" s="55"/>
+      <c r="N9" s="55"/>
+    </row>
+    <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="56" t="s">
+      <c r="C10" s="15"/>
+      <c r="D10" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="52" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" s="51"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="41"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="49"/>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="45" t="s">
+      <c r="E10" s="53" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="47"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="49"/>
-      <c r="M10" s="49"/>
-      <c r="N10" s="49"/>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="56"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="50"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="49"/>
-      <c r="L11" s="49"/>
-      <c r="M11" s="49"/>
-      <c r="N11" s="49"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="55"/>
+      <c r="N10" s="55"/>
+    </row>
+    <row r="11" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="16"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="67"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53"/>
+      <c r="J11" s="55"/>
+      <c r="K11" s="55"/>
+      <c r="L11" s="55"/>
+      <c r="M11" s="55"/>
+      <c r="N11" s="55"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="55" t="s">
+      <c r="B12" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="55"/>
-      <c r="D12" s="55"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
     </row>
     <row r="13" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="57"/>
-      <c r="F13" s="57"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="57"/>
-      <c r="K13" s="57"/>
-      <c r="L13" s="57"/>
-      <c r="M13" s="59" t="s">
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="40"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="60"/>
+      <c r="N13" s="42"/>
     </row>
     <row r="14" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="46" t="s">
+      <c r="B14" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24" t="s">
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="24"/>
+      <c r="I14" s="32"/>
       <c r="J14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="24" t="s">
+      <c r="K14" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="L14" s="25"/>
+      <c r="L14" s="33"/>
       <c r="M14" s="8" t="s">
         <v>19</v>
       </c>
@@ -1144,318 +1180,320 @@
       </c>
     </row>
     <row r="15" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="43"/>
+      <c r="K15" s="43"/>
+      <c r="L15" s="43"/>
       <c r="M15" s="1"/>
       <c r="N15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="33"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="36"/>
     </row>
     <row r="17" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="59" t="s">
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="57"/>
+      <c r="J17" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="K17" s="59"/>
-      <c r="L17" s="59"/>
-      <c r="M17" s="59" t="s">
+      <c r="K17" s="41"/>
+      <c r="L17" s="41"/>
+      <c r="M17" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="N17" s="59"/>
+      <c r="N17" s="41"/>
     </row>
     <row r="18" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
       <c r="F18" s="9" t="s">
         <v>28</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="30"/>
-      <c r="J18" s="26" t="s">
+      <c r="I18" s="54"/>
+      <c r="J18" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="26"/>
+      <c r="K18" s="27"/>
       <c r="L18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M18" s="27" t="s">
+      <c r="M18" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="N18" s="27"/>
+      <c r="N18" s="28"/>
     </row>
     <row r="19" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="28"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
       <c r="F19" s="9"/>
       <c r="G19" s="7"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="54"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
       <c r="L19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
     </row>
     <row r="20" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="28"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
       <c r="F20" s="9"/>
       <c r="G20" s="7"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="26"/>
-      <c r="K20" s="26"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="54"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
       <c r="L20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
     </row>
     <row r="21" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="28"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
       <c r="F21" s="9"/>
       <c r="G21" s="7"/>
-      <c r="H21" s="29"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="54"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
       <c r="L21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M21" s="27"/>
-      <c r="N21" s="27"/>
+      <c r="M21" s="28"/>
+      <c r="N21" s="28"/>
     </row>
     <row r="22" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
       <c r="F22" s="9"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="30"/>
-      <c r="J22" s="26"/>
-      <c r="K22" s="26"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="54"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
       <c r="L22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M22" s="27"/>
-      <c r="N22" s="27"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
     </row>
     <row r="23" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
       <c r="F23" s="9"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
       <c r="L23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
     </row>
     <row r="24" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
       <c r="F24" s="9"/>
       <c r="G24" s="7"/>
-      <c r="H24" s="29"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="54"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
       <c r="L24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
     </row>
     <row r="25" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="28"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
       <c r="F25" s="9"/>
       <c r="G25" s="7"/>
-      <c r="H25" s="29"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="54"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
       <c r="L25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M25" s="27"/>
-      <c r="N25" s="27"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
     </row>
     <row r="26" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
       <c r="F26" s="9"/>
       <c r="G26" s="7"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="54"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
       <c r="L26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
     </row>
     <row r="27" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
       <c r="F27" s="9"/>
       <c r="G27" s="7"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="54"/>
+      <c r="J27" s="27"/>
+      <c r="K27" s="27"/>
       <c r="L27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="19" t="s">
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
       <c r="N28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="18"/>
+      <c r="C30" s="22"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="D31" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="20" t="s">
         <v>36</v>
       </c>
       <c r="F31" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="H31" s="19">
+        <v>1</v>
+      </c>
+      <c r="I31" s="19"/>
+      <c r="J31" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="K31" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="L31" s="18" t="s">
         <v>39</v>
-      </c>
-      <c r="G31" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H31" s="15">
-        <v>1</v>
-      </c>
-      <c r="I31" s="15"/>
-      <c r="J31" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="K31" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="L31" s="14" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="D32" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32" s="17"/>
+        <v>40</v>
+      </c>
+      <c r="E32" s="21"/>
       <c r="F32" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G32" s="14"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="15"/>
-      <c r="L32" s="14"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="76">
-    <mergeCell ref="B6:C8"/>
-    <mergeCell ref="B9:C11"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="B27:E27"/>
+  <mergeCells count="78">
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="B17:I17"/>
@@ -1469,30 +1507,16 @@
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="E7:F8"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="J22:K22"/>
     <mergeCell ref="M7:N11"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="B8:C9"/>
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="K14:L14"/>
@@ -1506,10 +1530,9 @@
     <mergeCell ref="B15:L15"/>
     <mergeCell ref="G6:I6"/>
     <mergeCell ref="G7:I11"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="J21:K21"/>
@@ -1522,11 +1545,26 @@
     <mergeCell ref="J24:K24"/>
     <mergeCell ref="J25:K25"/>
     <mergeCell ref="B24:E24"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D10:D11"/>
     <mergeCell ref="L31:L32"/>
     <mergeCell ref="K31:K32"/>
     <mergeCell ref="E31:E32"/>
     <mergeCell ref="G31:G32"/>
     <mergeCell ref="H31:I32"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="H22:I22"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.75" header="0.1" footer="0.3"/>
   <pageSetup scale="74" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update(monitoring): update some of value to generate report
</commit_message>
<xml_diff>
--- a/src/lib/template/excel-template.xlsx
+++ b/src/lib/template/excel-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\TOHO(Fajar)\KCF\MC Monitoring System\kcf-mc-monitoring\src\lib\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103A4BE1-FA48-4A7A-9E2C-0AD2E0133893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E126845D-F5E9-4151-8E37-965F977C68B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A44CC11C-A6F5-42DE-B984-7CB6A06CB0CA}"/>
   </bookViews>
@@ -413,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -452,6 +452,60 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -463,6 +517,69 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -488,131 +605,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -971,28 +974,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
       <c r="H4" s="5" t="s">
         <v>20</v>
       </c>
@@ -1001,177 +1004,177 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="66" t="s">
+      <c r="C6" s="33"/>
+      <c r="D6" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="61" t="s">
+      <c r="E6" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="62"/>
-      <c r="G6" s="45" t="s">
+      <c r="F6" s="26"/>
+      <c r="G6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="46"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="34" t="s">
+      <c r="H6" s="48"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34" t="s">
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="N6" s="34"/>
+      <c r="N6" s="17"/>
     </row>
     <row r="7" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="53" t="s">
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="58"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
-      <c r="M7" s="55"/>
-      <c r="N7" s="55"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
     </row>
     <row r="8" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="66" t="s">
+      <c r="C8" s="33"/>
+      <c r="D8" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="64"/>
-      <c r="F8" s="65"/>
-      <c r="G8" s="48"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="55"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="50"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="52"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
     </row>
     <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="16"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="67"/>
-      <c r="E9" s="61" t="s">
+      <c r="B9" s="34"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="62"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="55"/>
-      <c r="K9" s="55"/>
-      <c r="L9" s="55"/>
-      <c r="M9" s="55"/>
-      <c r="N9" s="55"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
     </row>
     <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="66" t="s">
+      <c r="C10" s="33"/>
+      <c r="D10" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="53" t="s">
+      <c r="E10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="58"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="55"/>
-      <c r="K10" s="55"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="55"/>
-      <c r="N10" s="55"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="50"/>
+      <c r="H10" s="51"/>
+      <c r="I10" s="52"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
     </row>
     <row r="11" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="16"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="52"/>
-      <c r="I11" s="53"/>
-      <c r="J11" s="55"/>
-      <c r="K11" s="55"/>
-      <c r="L11" s="55"/>
-      <c r="M11" s="55"/>
-      <c r="N11" s="55"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="53"/>
+      <c r="H11" s="54"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="38"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="38"/>
-      <c r="M12" s="38"/>
-      <c r="N12" s="38"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+      <c r="K12" s="41"/>
+      <c r="L12" s="41"/>
+      <c r="M12" s="41"/>
+      <c r="N12" s="41"/>
     </row>
     <row r="13" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
-      <c r="J13" s="39"/>
-      <c r="K13" s="39"/>
-      <c r="L13" s="39"/>
-      <c r="M13" s="41" t="s">
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="42"/>
+      <c r="N13" s="44"/>
     </row>
     <row r="14" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32" t="s">
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="32"/>
+      <c r="I14" s="29"/>
       <c r="J14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="32" t="s">
+      <c r="K14" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="L14" s="33"/>
+      <c r="L14" s="37"/>
       <c r="M14" s="8" t="s">
         <v>19</v>
       </c>
@@ -1180,293 +1183,293 @@
       </c>
     </row>
     <row r="15" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="43"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="43"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
       <c r="M15" s="1"/>
       <c r="N15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35"/>
-      <c r="N16" s="36"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
+      <c r="N16" s="39"/>
     </row>
     <row r="17" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="56" t="s">
+      <c r="B17" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="57"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="41" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="K17" s="41"/>
-      <c r="L17" s="41"/>
-      <c r="M17" s="41" t="s">
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="N17" s="41"/>
+      <c r="N17" s="20"/>
     </row>
     <row r="18" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="29" t="s">
+      <c r="B18" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
       <c r="F18" s="9" t="s">
         <v>28</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="30" t="s">
+      <c r="H18" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="54"/>
-      <c r="J18" s="27" t="s">
+      <c r="I18" s="16"/>
+      <c r="J18" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="27"/>
+      <c r="K18" s="31"/>
       <c r="L18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M18" s="28" t="s">
+      <c r="M18" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="N18" s="28"/>
+      <c r="N18" s="55"/>
     </row>
     <row r="19" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
       <c r="F19" s="9"/>
       <c r="G19" s="7"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="54"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="27"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
       <c r="L19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
+      <c r="M19" s="55"/>
+      <c r="N19" s="55"/>
     </row>
     <row r="20" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="29"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
       <c r="F20" s="9"/>
       <c r="G20" s="7"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="54"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
       <c r="L20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
+      <c r="M20" s="55"/>
+      <c r="N20" s="55"/>
     </row>
     <row r="21" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="29"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
       <c r="F21" s="9"/>
       <c r="G21" s="7"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
       <c r="L21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M21" s="28"/>
-      <c r="N21" s="28"/>
+      <c r="M21" s="55"/>
+      <c r="N21" s="55"/>
     </row>
     <row r="22" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
       <c r="F22" s="9"/>
       <c r="G22" s="7"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="54"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
       <c r="L22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
+      <c r="M22" s="55"/>
+      <c r="N22" s="55"/>
     </row>
     <row r="23" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
       <c r="F23" s="9"/>
       <c r="G23" s="7"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="54"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
       <c r="L23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
+      <c r="M23" s="55"/>
+      <c r="N23" s="55"/>
     </row>
     <row r="24" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
       <c r="F24" s="9"/>
       <c r="G24" s="7"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="54"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
       <c r="L24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M24" s="28"/>
-      <c r="N24" s="28"/>
+      <c r="M24" s="55"/>
+      <c r="N24" s="55"/>
     </row>
     <row r="25" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="29"/>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
       <c r="F25" s="9"/>
       <c r="G25" s="7"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="27"/>
-      <c r="K25" s="27"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
       <c r="L25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
+      <c r="M25" s="55"/>
+      <c r="N25" s="55"/>
     </row>
     <row r="26" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
       <c r="F26" s="9"/>
       <c r="G26" s="7"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="54"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
       <c r="L26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M26" s="28"/>
-      <c r="N26" s="28"/>
+      <c r="M26" s="55"/>
+      <c r="N26" s="55"/>
     </row>
     <row r="27" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="29"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
       <c r="F27" s="9"/>
       <c r="G27" s="7"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="54"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
       <c r="L27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M27" s="28"/>
-      <c r="N27" s="28"/>
+      <c r="M27" s="55"/>
+      <c r="N27" s="55"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B28" s="25" t="s">
+      <c r="B28" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="25"/>
-      <c r="J28" s="23" t="s">
+      <c r="C28" s="64"/>
+      <c r="D28" s="64"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="64"/>
+      <c r="G28" s="64"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="64"/>
+      <c r="J28" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="K28" s="24"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24"/>
+      <c r="K28" s="63"/>
+      <c r="L28" s="63"/>
+      <c r="M28" s="63"/>
       <c r="N28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="61" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="22"/>
+      <c r="C30" s="61"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="D31" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="59" t="s">
         <v>36</v>
       </c>
       <c r="F31" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="H31" s="19">
+      <c r="H31" s="58">
         <v>1</v>
       </c>
-      <c r="I31" s="19"/>
-      <c r="J31" s="21" t="s">
+      <c r="I31" s="58"/>
+      <c r="J31" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="K31" s="19" t="s">
+      <c r="K31" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="L31" s="18" t="s">
+      <c r="L31" s="57" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1474,26 +1477,73 @@
       <c r="D32" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E32" s="21"/>
+      <c r="E32" s="60"/>
       <c r="F32" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G32" s="18"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="18"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="58"/>
+      <c r="I32" s="58"/>
+      <c r="J32" s="60"/>
+      <c r="K32" s="58"/>
+      <c r="L32" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H31:I32"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="B2:N2"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B12:N12"/>
+    <mergeCell ref="B13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I11"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M7:N11"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="B8:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D10:D11"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="B17:I17"/>
@@ -1510,61 +1560,14 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="E7:F8"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
     <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M7:N11"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="B6:C7"/>
-    <mergeCell ref="B8:C9"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="B16:N16"/>
-    <mergeCell ref="B12:N12"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B15:L15"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I11"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:I32"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="H22:I22"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.75" header="0.1" footer="0.3"/>
   <pageSetup scale="74" orientation="portrait" r:id="rId1"/>
@@ -1698,18 +1701,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1731,14 +1734,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14EA48F8-1535-4600-B361-5A56BC1EA18D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="b7409cf6-e852-4a78-b0e6-5ba582a53027"/>
@@ -1752,4 +1747,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
misc: update template columns, product rpm null handling, card sizing
- fill-template.ts: update all column mappings (dandori B/J/N/O/Q/R,
  production B/G/H/J/L/N/P/Q with Status at L, problem B/E/F/G/H/I/J)
  to match new Excel template layout
- excel-template.xlsx: updated template with new column structure
- monitoring page: keep CYOKOTEI_STOP in production entries alongside
  problem entries (not mutually exclusive)
- product-model.ts: add | null to rpm type in ProductData,
  ProductUpdatePayload, ProductCreatePayload
- ProductUpdateModal: parse RPM string to number, handle NaN as null
- MachineCardCompact: enlarge text (xs→lg), icons (size-3→size-6),
  add py-1 padding to card
</commit_message>
<xml_diff>
--- a/src/lib/template/excel-template.xlsx
+++ b/src/lib/template/excel-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\TOHO(Fajar)\KCF\MC Monitoring System\kcf-mc-monitoring\src\lib\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E126845D-F5E9-4151-8E37-965F977C68B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B666E708-0E88-4724-90B2-7D9205F0296A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A44CC11C-A6F5-42DE-B984-7CB6A06CB0CA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="54">
   <si>
     <t>Part Name</t>
   </si>
@@ -171,6 +171,36 @@
   </si>
   <si>
     <t>{{Customer}}</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>{{Status}}</t>
+  </si>
+  <si>
+    <t>PROBLEM</t>
+  </si>
+  <si>
+    <t>KAIZEN</t>
+  </si>
+  <si>
+    <t>PENANGANAN</t>
+  </si>
+  <si>
+    <t>{{ProblemDate}}</t>
+  </si>
+  <si>
+    <t>{{ProblemStart}}</t>
+  </si>
+  <si>
+    <t>{{ProblemEnd}}</t>
+  </si>
+  <si>
+    <t>{{ProblemPIC}}</t>
+  </si>
+  <si>
+    <t>{{ProblemDuration}}</t>
   </si>
 </sst>
 </file>
@@ -413,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -428,9 +458,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -444,13 +471,84 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -458,32 +556,170 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -491,131 +727,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -954,627 +1085,1041 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N32"/>
+  <dimension ref="B2:R42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="6.5703125" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="2.85546875" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="3.140625" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="3" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="17" customWidth="1"/>
-    <col min="14" max="14" width="5.42578125" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="6" max="6" width="2.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="8" max="8" width="6.5703125" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" customWidth="1"/>
+    <col min="11" max="11" width="7.140625" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" customWidth="1"/>
+    <col min="13" max="13" width="6.28515625" customWidth="1"/>
+    <col min="14" max="14" width="3" customWidth="1"/>
+    <col min="15" max="15" width="16.140625" customWidth="1"/>
+    <col min="16" max="16" width="4.7109375" customWidth="1"/>
+    <col min="17" max="17" width="14.42578125" customWidth="1"/>
+    <col min="18" max="18" width="5.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="36" t="s">
+    <row r="2" spans="2:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="56" t="s">
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+    </row>
+    <row r="4" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B4" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="H4" s="5" t="s">
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="12"/>
+      <c r="J4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="K4" s="48" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="32" t="s">
+      <c r="L4" s="48"/>
+      <c r="M4" s="48"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="15"/>
+    </row>
+    <row r="6" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="30" t="s">
+      <c r="C6" s="45"/>
+      <c r="D6" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="65"/>
+      <c r="F6" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="26"/>
-      <c r="G6" s="47" t="s">
+      <c r="G6" s="99"/>
+      <c r="H6" s="100"/>
+      <c r="I6" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="48"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="17" t="s">
+      <c r="J6" s="87"/>
+      <c r="K6" s="87"/>
+      <c r="L6" s="87"/>
+      <c r="M6" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17" t="s">
+      <c r="N6" s="64"/>
+      <c r="O6" s="64"/>
+      <c r="P6" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="N6" s="17"/>
-    </row>
-    <row r="7" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="34"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="65" t="s">
+      <c r="Q6" s="72"/>
+      <c r="R6" s="73"/>
+    </row>
+    <row r="7" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="46"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="90"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="66"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="27"/>
-      <c r="M7" s="27"/>
-      <c r="N7" s="27"/>
-    </row>
-    <row r="8" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="32" t="s">
+      <c r="G7" s="102"/>
+      <c r="H7" s="103"/>
+      <c r="I7" s="85"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="66"/>
+      <c r="P7" s="74"/>
+      <c r="Q7" s="75"/>
+      <c r="R7" s="76"/>
+    </row>
+    <row r="8" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="30" t="s">
+      <c r="C8" s="45"/>
+      <c r="D8" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="67"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="51"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
-      <c r="N8" s="27"/>
-    </row>
-    <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="34"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="25" t="s">
+      <c r="E8" s="65"/>
+      <c r="F8" s="104"/>
+      <c r="G8" s="105"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="85"/>
+      <c r="J8" s="85"/>
+      <c r="K8" s="85"/>
+      <c r="L8" s="85"/>
+      <c r="M8" s="67"/>
+      <c r="N8" s="67"/>
+      <c r="O8" s="68"/>
+      <c r="P8" s="77"/>
+      <c r="Q8" s="78"/>
+      <c r="R8" s="79"/>
+    </row>
+    <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="46"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="98" t="s">
         <v>2</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="52"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-    </row>
-    <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="32" t="s">
+      <c r="G9" s="99"/>
+      <c r="H9" s="100"/>
+      <c r="I9" s="85"/>
+      <c r="J9" s="85"/>
+      <c r="K9" s="85"/>
+      <c r="L9" s="85"/>
+      <c r="M9" s="67"/>
+      <c r="N9" s="67"/>
+      <c r="O9" s="68"/>
+      <c r="P9" s="77"/>
+      <c r="Q9" s="78"/>
+      <c r="R9" s="79"/>
+    </row>
+    <row r="10" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="30" t="s">
+      <c r="C10" s="45"/>
+      <c r="D10" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="E10" s="67"/>
+      <c r="F10" s="91" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="22"/>
-      <c r="G10" s="50"/>
-      <c r="H10" s="51"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="27"/>
-      <c r="M10" s="27"/>
-      <c r="N10" s="27"/>
-    </row>
-    <row r="11" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="34"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="27"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="40" t="s">
+      <c r="G10" s="67"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="85"/>
+      <c r="J10" s="85"/>
+      <c r="K10" s="85"/>
+      <c r="L10" s="85"/>
+      <c r="M10" s="67"/>
+      <c r="N10" s="67"/>
+      <c r="O10" s="68"/>
+      <c r="P10" s="77"/>
+      <c r="Q10" s="78"/>
+      <c r="R10" s="79"/>
+    </row>
+    <row r="11" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="46"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="90"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="70"/>
+      <c r="I11" s="85"/>
+      <c r="J11" s="85"/>
+      <c r="K11" s="85"/>
+      <c r="L11" s="85"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="O11" s="70"/>
+      <c r="P11" s="80"/>
+      <c r="Q11" s="81"/>
+      <c r="R11" s="82"/>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
-      <c r="N12" s="41"/>
-    </row>
-    <row r="13" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="42" t="s">
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="35"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="35"/>
+      <c r="N12" s="35"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="35"/>
+      <c r="Q12" s="35"/>
+      <c r="R12" s="35"/>
+    </row>
+    <row r="13" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="42"/>
-      <c r="M13" s="20" t="s">
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="37"/>
+      <c r="M13" s="37"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+      <c r="P13" s="36"/>
+      <c r="Q13" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="44"/>
-    </row>
-    <row r="14" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="28" t="s">
+      <c r="R13" s="39"/>
+    </row>
+    <row r="14" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29" t="s">
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="29"/>
-      <c r="J14" s="7" t="s">
+      <c r="K14" s="28"/>
+      <c r="L14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="N14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K14" s="29" t="s">
+      <c r="O14" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="L14" s="37"/>
-      <c r="M14" s="8" t="s">
+      <c r="P14" s="29"/>
+      <c r="Q14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="N14" s="3" t="s">
+      <c r="R14" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="4" t="s">
+    <row r="15" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+      <c r="N15" s="40"/>
+      <c r="O15" s="40"/>
+      <c r="P15" s="40"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="38" t="s">
+    <row r="16" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="38"/>
-      <c r="N16" s="39"/>
-    </row>
-    <row r="17" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="s">
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="32"/>
+      <c r="R16" s="33"/>
+    </row>
+    <row r="17" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="20" t="s">
+      <c r="C17" s="62"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="62"/>
+      <c r="J17" s="62"/>
+      <c r="K17" s="63"/>
+      <c r="L17" s="83" t="s">
+        <v>44</v>
+      </c>
+      <c r="M17" s="83"/>
+      <c r="N17" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-      <c r="M17" s="20" t="s">
+      <c r="O17" s="38"/>
+      <c r="P17" s="38"/>
+      <c r="Q17" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="N17" s="20"/>
-    </row>
-    <row r="18" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="14" t="s">
+      <c r="R17" s="38"/>
+    </row>
+    <row r="18" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="9" t="s">
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="H18" s="97" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="I18" s="97"/>
+      <c r="J18" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="31" t="s">
+      <c r="K18" s="43"/>
+      <c r="L18" s="84" t="s">
+        <v>45</v>
+      </c>
+      <c r="M18" s="84"/>
+      <c r="N18" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="K18" s="31"/>
-      <c r="L18" s="4" t="s">
+      <c r="O18" s="31"/>
+      <c r="P18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M18" s="55" t="s">
+      <c r="Q18" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="N18" s="55"/>
-    </row>
-    <row r="19" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="14"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="4" t="s">
+      <c r="R18" s="26"/>
+    </row>
+    <row r="19" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="42"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="97"/>
+      <c r="I19" s="97"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="43"/>
+      <c r="L19" s="84"/>
+      <c r="M19" s="84"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="31"/>
+      <c r="P19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M19" s="55"/>
-      <c r="N19" s="55"/>
-    </row>
-    <row r="20" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="14"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="4" t="s">
+      <c r="Q19" s="26"/>
+      <c r="R19" s="26"/>
+    </row>
+    <row r="20" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="42"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="97"/>
+      <c r="I20" s="97"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="84"/>
+      <c r="M20" s="84"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="31"/>
+      <c r="P20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M20" s="55"/>
-      <c r="N20" s="55"/>
-    </row>
-    <row r="21" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="14"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="4" t="s">
+      <c r="Q20" s="26"/>
+      <c r="R20" s="26"/>
+    </row>
+    <row r="21" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="97"/>
+      <c r="I21" s="97"/>
+      <c r="J21" s="43"/>
+      <c r="K21" s="43"/>
+      <c r="L21" s="84"/>
+      <c r="M21" s="84"/>
+      <c r="N21" s="30"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M21" s="55"/>
-      <c r="N21" s="55"/>
-    </row>
-    <row r="22" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="14"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="4" t="s">
+      <c r="Q21" s="26"/>
+      <c r="R21" s="26"/>
+    </row>
+    <row r="22" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="42"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="97"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="43"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="84"/>
+      <c r="N22" s="30"/>
+      <c r="O22" s="31"/>
+      <c r="P22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M22" s="55"/>
-      <c r="N22" s="55"/>
-    </row>
-    <row r="23" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="14"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="4" t="s">
+      <c r="Q22" s="26"/>
+      <c r="R22" s="26"/>
+    </row>
+    <row r="23" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="42"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="97"/>
+      <c r="I23" s="97"/>
+      <c r="J23" s="43"/>
+      <c r="K23" s="43"/>
+      <c r="L23" s="84"/>
+      <c r="M23" s="84"/>
+      <c r="N23" s="30"/>
+      <c r="O23" s="31"/>
+      <c r="P23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M23" s="55"/>
-      <c r="N23" s="55"/>
-    </row>
-    <row r="24" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="14"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="31"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="4" t="s">
+      <c r="Q23" s="26"/>
+      <c r="R23" s="26"/>
+    </row>
+    <row r="24" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="42"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="97"/>
+      <c r="I24" s="97"/>
+      <c r="J24" s="43"/>
+      <c r="K24" s="43"/>
+      <c r="L24" s="84"/>
+      <c r="M24" s="84"/>
+      <c r="N24" s="30"/>
+      <c r="O24" s="31"/>
+      <c r="P24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M24" s="55"/>
-      <c r="N24" s="55"/>
-    </row>
-    <row r="25" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="14"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="4" t="s">
+      <c r="Q24" s="26"/>
+      <c r="R24" s="26"/>
+    </row>
+    <row r="25" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="42"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="97"/>
+      <c r="I25" s="97"/>
+      <c r="J25" s="43"/>
+      <c r="K25" s="43"/>
+      <c r="L25" s="84"/>
+      <c r="M25" s="84"/>
+      <c r="N25" s="30"/>
+      <c r="O25" s="31"/>
+      <c r="P25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M25" s="55"/>
-      <c r="N25" s="55"/>
-    </row>
-    <row r="26" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="14"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="31"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="4" t="s">
+      <c r="Q25" s="26"/>
+      <c r="R25" s="26"/>
+    </row>
+    <row r="26" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="42"/>
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="97"/>
+      <c r="I26" s="97"/>
+      <c r="J26" s="43"/>
+      <c r="K26" s="43"/>
+      <c r="L26" s="84"/>
+      <c r="M26" s="84"/>
+      <c r="N26" s="30"/>
+      <c r="O26" s="31"/>
+      <c r="P26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M26" s="55"/>
-      <c r="N26" s="55"/>
-    </row>
-    <row r="27" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="14"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="4" t="s">
+      <c r="Q26" s="26"/>
+      <c r="R26" s="26"/>
+    </row>
+    <row r="27" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="42"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="97"/>
+      <c r="I27" s="97"/>
+      <c r="J27" s="43"/>
+      <c r="K27" s="43"/>
+      <c r="L27" s="84"/>
+      <c r="M27" s="84"/>
+      <c r="N27" s="30"/>
+      <c r="O27" s="31"/>
+      <c r="P27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M27" s="55"/>
-      <c r="N27" s="55"/>
-    </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B28" s="64" t="s">
+      <c r="Q27" s="26"/>
+      <c r="R27" s="26"/>
+    </row>
+    <row r="28" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B28" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="64"/>
-      <c r="D28" s="64"/>
-      <c r="E28" s="64"/>
-      <c r="F28" s="64"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="64"/>
-      <c r="J28" s="62" t="s">
+      <c r="C28" s="95"/>
+      <c r="D28" s="95"/>
+      <c r="E28" s="95"/>
+      <c r="F28" s="95"/>
+      <c r="G28" s="95"/>
+      <c r="H28" s="95"/>
+      <c r="I28" s="95"/>
+      <c r="J28" s="95"/>
+      <c r="K28" s="95"/>
+      <c r="L28" s="95"/>
+      <c r="M28" s="95"/>
+      <c r="N28" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="K28" s="63"/>
-      <c r="L28" s="63"/>
-      <c r="M28" s="63"/>
-      <c r="N28" s="2" t="s">
+      <c r="O28" s="93"/>
+      <c r="P28" s="93"/>
+      <c r="Q28" s="93"/>
+      <c r="R28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="61" t="s">
+    <row r="29" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B29" s="16"/>
+      <c r="C29" s="17"/>
+      <c r="R29" s="21"/>
+    </row>
+    <row r="30" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B30" s="94" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="61"/>
-    </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="D31" s="10" t="s">
+      <c r="C30" s="54"/>
+      <c r="R30" s="22"/>
+    </row>
+    <row r="31" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B31" s="18"/>
+      <c r="D31" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E31" s="59" t="s">
+      <c r="E31" s="14"/>
+      <c r="F31" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="G31" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="G31" s="57" t="s">
+      <c r="H31" s="54"/>
+      <c r="I31" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="H31" s="58">
+      <c r="J31" s="49">
         <v>1</v>
       </c>
-      <c r="I31" s="58"/>
-      <c r="J31" s="60" t="s">
+      <c r="K31" s="49"/>
+      <c r="L31" s="49"/>
+      <c r="M31" s="49"/>
+      <c r="N31" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="K31" s="58" t="s">
+      <c r="O31" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="L31" s="57" t="s">
+      <c r="P31" s="48" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="D32" s="12" t="s">
+      <c r="R31" s="22"/>
+    </row>
+    <row r="32" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B32" s="18"/>
+      <c r="D32" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E32" s="60"/>
-      <c r="F32" s="11" t="s">
+      <c r="E32" s="14"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="54" t="s">
         <v>35</v>
       </c>
-      <c r="G32" s="57"/>
-      <c r="H32" s="58"/>
-      <c r="I32" s="58"/>
-      <c r="J32" s="60"/>
-      <c r="K32" s="58"/>
-      <c r="L32" s="57"/>
+      <c r="H32" s="54"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+      <c r="M32" s="49"/>
+      <c r="N32" s="51"/>
+      <c r="O32" s="49"/>
+      <c r="P32" s="48"/>
+      <c r="R32" s="22"/>
+    </row>
+    <row r="33" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B33" s="19"/>
+      <c r="C33" s="20"/>
+      <c r="R33" s="23"/>
+    </row>
+    <row r="34" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B34" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="32"/>
+      <c r="J34" s="32"/>
+      <c r="K34" s="32"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+      <c r="O34" s="32"/>
+      <c r="P34" s="32"/>
+      <c r="Q34" s="32"/>
+      <c r="R34" s="32"/>
+    </row>
+    <row r="35" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B35" s="56" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="57"/>
+      <c r="D35" s="57"/>
+      <c r="E35" s="57"/>
+      <c r="F35" s="57"/>
+      <c r="G35" s="58"/>
+      <c r="H35" s="59" t="s">
+        <v>8</v>
+      </c>
+      <c r="I35" s="60"/>
+      <c r="J35" s="56" t="s">
+        <v>12</v>
+      </c>
+      <c r="K35" s="58"/>
+      <c r="L35" s="56" t="s">
+        <v>48</v>
+      </c>
+      <c r="M35" s="57"/>
+      <c r="N35" s="57"/>
+      <c r="O35" s="58"/>
+      <c r="P35" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q35" s="55"/>
+      <c r="R35" s="55"/>
+    </row>
+    <row r="36" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B36" s="92" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="93"/>
+      <c r="D36" s="93"/>
+      <c r="E36" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H36" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="I36" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J36" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="K36" s="96"/>
+      <c r="L36" s="30"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
+      <c r="O36" s="96"/>
+      <c r="P36" s="30"/>
+      <c r="Q36" s="31"/>
+      <c r="R36" s="96"/>
+    </row>
+    <row r="37" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="46"/>
+      <c r="C37" s="88"/>
+      <c r="D37" s="88"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J37" s="31"/>
+      <c r="K37" s="96"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
+      <c r="O37" s="96"/>
+      <c r="P37" s="30"/>
+      <c r="Q37" s="31"/>
+      <c r="R37" s="96"/>
+    </row>
+    <row r="38" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="46"/>
+      <c r="C38" s="88"/>
+      <c r="D38" s="88"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="25"/>
+      <c r="I38" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J38" s="31"/>
+      <c r="K38" s="96"/>
+      <c r="L38" s="30"/>
+      <c r="M38" s="31"/>
+      <c r="N38" s="31"/>
+      <c r="O38" s="96"/>
+      <c r="P38" s="30"/>
+      <c r="Q38" s="31"/>
+      <c r="R38" s="96"/>
+    </row>
+    <row r="39" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="46"/>
+      <c r="C39" s="88"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J39" s="31"/>
+      <c r="K39" s="96"/>
+      <c r="L39" s="30"/>
+      <c r="M39" s="31"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="96"/>
+      <c r="P39" s="30"/>
+      <c r="Q39" s="31"/>
+      <c r="R39" s="96"/>
+    </row>
+    <row r="40" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="46"/>
+      <c r="C40" s="88"/>
+      <c r="D40" s="88"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J40" s="31"/>
+      <c r="K40" s="96"/>
+      <c r="L40" s="30"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="31"/>
+      <c r="O40" s="96"/>
+      <c r="P40" s="30"/>
+      <c r="Q40" s="31"/>
+      <c r="R40" s="96"/>
+    </row>
+    <row r="41" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="46"/>
+      <c r="C41" s="88"/>
+      <c r="D41" s="88"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="25"/>
+      <c r="I41" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J41" s="31"/>
+      <c r="K41" s="96"/>
+      <c r="L41" s="30"/>
+      <c r="M41" s="31"/>
+      <c r="N41" s="31"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="30"/>
+      <c r="Q41" s="31"/>
+      <c r="R41" s="96"/>
+    </row>
+    <row r="42" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="46"/>
+      <c r="C42" s="88"/>
+      <c r="D42" s="88"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="107" t="s">
+        <v>9</v>
+      </c>
+      <c r="J42" s="31"/>
+      <c r="K42" s="96"/>
+      <c r="L42" s="30"/>
+      <c r="M42" s="31"/>
+      <c r="N42" s="31"/>
+      <c r="O42" s="96"/>
+      <c r="P42" s="30"/>
+      <c r="Q42" s="31"/>
+      <c r="R42" s="96"/>
     </row>
   </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="J23:K23"/>
+  <mergeCells count="136">
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="N28:Q28"/>
+    <mergeCell ref="P41:R41"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H21:I21"/>
     <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="P36:R36"/>
+    <mergeCell ref="P37:R37"/>
+    <mergeCell ref="P38:R38"/>
+    <mergeCell ref="P39:R39"/>
+    <mergeCell ref="P40:R40"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="D8:E9"/>
+    <mergeCell ref="D10:E11"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B35:G35"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:I32"/>
+    <mergeCell ref="B28:M28"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F7:H8"/>
+    <mergeCell ref="F10:H11"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="L40:O40"/>
+    <mergeCell ref="L41:O41"/>
+    <mergeCell ref="L42:O42"/>
+    <mergeCell ref="L36:O36"/>
+    <mergeCell ref="L37:O37"/>
+    <mergeCell ref="P35:R35"/>
+    <mergeCell ref="L35:O35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B34:R34"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="M7:O11"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="I7:L11"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:M32"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="B27:F27"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B25:F25"/>
     <mergeCell ref="J26:K26"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="B2:N2"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="B16:N16"/>
-    <mergeCell ref="B12:N12"/>
-    <mergeCell ref="B13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B15:L15"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I11"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M7:N11"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="B16:R16"/>
+    <mergeCell ref="B12:R12"/>
+    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="B15:P15"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="B6:C7"/>
     <mergeCell ref="B8:C9"/>
     <mergeCell ref="B10:C11"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="E10:F11"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="J7:L11"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="E7:F8"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.75" header="0.1" footer="0.3"/>
-  <pageSetup scale="74" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="71" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007BE2B6646B9ABC4BB267BAC3E807C6E7" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5fc71d7168c8e25ad2b9f4649bdf9088">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b7409cf6-e852-4a78-b0e6-5ba582a53027" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="176a8bbe9a0b68c96965844395333f21" ns3:_="">
     <xsd:import namespace="b7409cf6-e852-4a78-b0e6-5ba582a53027"/>
@@ -1700,22 +2245,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14EA48F8-1535-4600-B361-5A56BC1EA18D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="b7409cf6-e852-4a78-b0e6-5ba582a53027"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8EB11ABF-3551-440C-B418-2A20E9C4FC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1731,28 +2285,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14EA48F8-1535-4600-B361-5A56BC1EA18D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="b7409cf6-e852-4a78-b0e6-5ba582a53027"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update(template): update excel template
</commit_message>
<xml_diff>
--- a/src/lib/template/excel-template.xlsx
+++ b/src/lib/template/excel-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\TOHO(Fajar)\KCF\MC Monitoring System\kcf-mc-monitoring\src\lib\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B666E708-0E88-4724-90B2-7D9205F0296A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B10AE0E-F196-4556-B802-E41E9CBF038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A44CC11C-A6F5-42DE-B984-7CB6A06CB0CA}"/>
   </bookViews>
@@ -443,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -502,27 +502,216 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -550,203 +739,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1109,252 +1112,252 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="94" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
-      <c r="O2" s="27"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="94"/>
+      <c r="R2" s="94"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
       <c r="E4" s="12"/>
       <c r="J4" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="48" t="s">
+      <c r="K4" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
       <c r="O4" s="15"/>
     </row>
     <row r="6" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="105" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="45"/>
-      <c r="D6" s="89" t="s">
+      <c r="C6" s="106"/>
+      <c r="D6" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="65"/>
-      <c r="F6" s="98" t="s">
+      <c r="E6" s="37"/>
+      <c r="F6" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="99"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="86" t="s">
+      <c r="G6" s="49"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="J6" s="87"/>
-      <c r="K6" s="87"/>
-      <c r="L6" s="87"/>
-      <c r="M6" s="64" t="s">
+      <c r="J6" s="85"/>
+      <c r="K6" s="85"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="N6" s="64"/>
-      <c r="O6" s="64"/>
-      <c r="P6" s="71" t="s">
+      <c r="N6" s="67"/>
+      <c r="O6" s="67"/>
+      <c r="P6" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="Q6" s="72"/>
-      <c r="R6" s="73"/>
+      <c r="Q6" s="70"/>
+      <c r="R6" s="71"/>
     </row>
     <row r="7" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="46"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="90"/>
-      <c r="E7" s="69"/>
-      <c r="F7" s="101" t="s">
+      <c r="B7" s="34"/>
+      <c r="C7" s="107"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="102"/>
-      <c r="H7" s="103"/>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
-      <c r="L7" s="85"/>
-      <c r="M7" s="65"/>
-      <c r="N7" s="65"/>
-      <c r="O7" s="66"/>
-      <c r="P7" s="74"/>
-      <c r="Q7" s="75"/>
-      <c r="R7" s="76"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="53"/>
+      <c r="I7" s="83"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="83"/>
+      <c r="L7" s="83"/>
+      <c r="M7" s="37"/>
+      <c r="N7" s="37"/>
+      <c r="O7" s="68"/>
+      <c r="P7" s="72"/>
+      <c r="Q7" s="73"/>
+      <c r="R7" s="74"/>
     </row>
     <row r="8" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="105" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="45"/>
-      <c r="D8" s="89" t="s">
+      <c r="C8" s="106"/>
+      <c r="D8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="65"/>
-      <c r="F8" s="104"/>
-      <c r="G8" s="105"/>
-      <c r="H8" s="106"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="85"/>
-      <c r="K8" s="85"/>
-      <c r="L8" s="85"/>
-      <c r="M8" s="67"/>
-      <c r="N8" s="67"/>
-      <c r="O8" s="68"/>
-      <c r="P8" s="77"/>
-      <c r="Q8" s="78"/>
-      <c r="R8" s="79"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="83"/>
+      <c r="J8" s="83"/>
+      <c r="K8" s="83"/>
+      <c r="L8" s="83"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="57"/>
+      <c r="P8" s="75"/>
+      <c r="Q8" s="76"/>
+      <c r="R8" s="77"/>
     </row>
     <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="46"/>
-      <c r="C9" s="47"/>
-      <c r="D9" s="91"/>
-      <c r="E9" s="67"/>
-      <c r="F9" s="98" t="s">
+      <c r="B9" s="34"/>
+      <c r="C9" s="107"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="99"/>
-      <c r="H9" s="100"/>
-      <c r="I9" s="85"/>
-      <c r="J9" s="85"/>
-      <c r="K9" s="85"/>
-      <c r="L9" s="85"/>
-      <c r="M9" s="67"/>
-      <c r="N9" s="67"/>
-      <c r="O9" s="68"/>
-      <c r="P9" s="77"/>
-      <c r="Q9" s="78"/>
-      <c r="R9" s="79"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="83"/>
+      <c r="J9" s="83"/>
+      <c r="K9" s="83"/>
+      <c r="L9" s="83"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="57"/>
+      <c r="P9" s="75"/>
+      <c r="Q9" s="76"/>
+      <c r="R9" s="77"/>
     </row>
     <row r="10" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="C10" s="45"/>
-      <c r="D10" s="91" t="s">
+      <c r="C10" s="106"/>
+      <c r="D10" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="67"/>
-      <c r="F10" s="91" t="s">
+      <c r="E10" s="41"/>
+      <c r="F10" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="67"/>
-      <c r="H10" s="68"/>
-      <c r="I10" s="85"/>
-      <c r="J10" s="85"/>
-      <c r="K10" s="85"/>
-      <c r="L10" s="85"/>
-      <c r="M10" s="67"/>
-      <c r="N10" s="67"/>
-      <c r="O10" s="68"/>
-      <c r="P10" s="77"/>
-      <c r="Q10" s="78"/>
-      <c r="R10" s="79"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="83"/>
+      <c r="K10" s="83"/>
+      <c r="L10" s="83"/>
+      <c r="M10" s="41"/>
+      <c r="N10" s="41"/>
+      <c r="O10" s="57"/>
+      <c r="P10" s="75"/>
+      <c r="Q10" s="76"/>
+      <c r="R10" s="77"/>
     </row>
     <row r="11" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="46"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="69"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="70"/>
-      <c r="I11" s="85"/>
-      <c r="J11" s="85"/>
-      <c r="K11" s="85"/>
-      <c r="L11" s="85"/>
-      <c r="M11" s="69"/>
-      <c r="N11" s="69"/>
-      <c r="O11" s="70"/>
-      <c r="P11" s="80"/>
-      <c r="Q11" s="81"/>
-      <c r="R11" s="82"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="107"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="58"/>
+      <c r="I11" s="83"/>
+      <c r="J11" s="83"/>
+      <c r="K11" s="83"/>
+      <c r="L11" s="83"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="58"/>
+      <c r="P11" s="78"/>
+      <c r="Q11" s="79"/>
+      <c r="R11" s="80"/>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="97" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="35"/>
-      <c r="P12" s="35"/>
-      <c r="Q12" s="35"/>
-      <c r="R12" s="35"/>
+      <c r="C12" s="97"/>
+      <c r="D12" s="97"/>
+      <c r="E12" s="97"/>
+      <c r="F12" s="98"/>
+      <c r="G12" s="98"/>
+      <c r="H12" s="98"/>
+      <c r="I12" s="98"/>
+      <c r="J12" s="98"/>
+      <c r="K12" s="98"/>
+      <c r="L12" s="98"/>
+      <c r="M12" s="98"/>
+      <c r="N12" s="98"/>
+      <c r="O12" s="98"/>
+      <c r="P12" s="98"/>
+      <c r="Q12" s="98"/>
+      <c r="R12" s="98"/>
     </row>
     <row r="13" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="99" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="36"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
-      <c r="L13" s="37"/>
-      <c r="M13" s="37"/>
-      <c r="N13" s="36"/>
-      <c r="O13" s="36"/>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="38" t="s">
+      <c r="C13" s="99"/>
+      <c r="D13" s="99"/>
+      <c r="E13" s="99"/>
+      <c r="F13" s="99"/>
+      <c r="G13" s="99"/>
+      <c r="H13" s="99"/>
+      <c r="I13" s="99"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
+      <c r="N13" s="99"/>
+      <c r="O13" s="99"/>
+      <c r="P13" s="99"/>
+      <c r="Q13" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="R13" s="39"/>
+      <c r="R13" s="102"/>
     </row>
     <row r="14" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28" t="s">
+      <c r="C14" s="92"/>
+      <c r="D14" s="92"/>
+      <c r="E14" s="92"/>
+      <c r="F14" s="92"/>
+      <c r="G14" s="92"/>
+      <c r="H14" s="92"/>
+      <c r="I14" s="92"/>
+      <c r="J14" s="92" t="s">
         <v>25</v>
       </c>
-      <c r="K14" s="28"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="28"/>
+      <c r="K14" s="92"/>
+      <c r="L14" s="92"/>
+      <c r="M14" s="92"/>
       <c r="N14" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="O14" s="28" t="s">
+      <c r="O14" s="92" t="s">
         <v>26</v>
       </c>
-      <c r="P14" s="29"/>
+      <c r="P14" s="95"/>
       <c r="Q14" s="7" t="s">
         <v>19</v>
       </c>
@@ -1363,319 +1366,319 @@
       </c>
     </row>
     <row r="15" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="41"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
+      <c r="B15" s="103"/>
+      <c r="C15" s="103"/>
+      <c r="D15" s="103"/>
+      <c r="E15" s="103"/>
+      <c r="F15" s="103"/>
+      <c r="G15" s="103"/>
+      <c r="H15" s="103"/>
+      <c r="I15" s="103"/>
+      <c r="J15" s="104"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="104"/>
+      <c r="M15" s="104"/>
+      <c r="N15" s="103"/>
+      <c r="O15" s="103"/>
+      <c r="P15" s="103"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
-      <c r="L16" s="32"/>
-      <c r="M16" s="32"/>
-      <c r="N16" s="32"/>
-      <c r="O16" s="32"/>
-      <c r="P16" s="32"/>
-      <c r="Q16" s="32"/>
-      <c r="R16" s="33"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
+      <c r="G16" s="66"/>
+      <c r="H16" s="66"/>
+      <c r="I16" s="66"/>
+      <c r="J16" s="66"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="66"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="66"/>
+      <c r="O16" s="66"/>
+      <c r="P16" s="66"/>
+      <c r="Q16" s="66"/>
+      <c r="R16" s="96"/>
     </row>
     <row r="17" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="C17" s="62"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-      <c r="I17" s="62"/>
-      <c r="J17" s="62"/>
-      <c r="K17" s="63"/>
-      <c r="L17" s="83" t="s">
+      <c r="C17" s="64"/>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="64"/>
+      <c r="H17" s="64"/>
+      <c r="I17" s="64"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="65"/>
+      <c r="L17" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="M17" s="83"/>
-      <c r="N17" s="38" t="s">
+      <c r="M17" s="81"/>
+      <c r="N17" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="O17" s="38"/>
-      <c r="P17" s="38"/>
-      <c r="Q17" s="38" t="s">
+      <c r="O17" s="108"/>
+      <c r="P17" s="108"/>
+      <c r="Q17" s="108" t="s">
         <v>12</v>
       </c>
-      <c r="R17" s="38"/>
+      <c r="R17" s="108"/>
     </row>
     <row r="18" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
+      <c r="C18" s="89"/>
+      <c r="D18" s="89"/>
+      <c r="E18" s="89"/>
+      <c r="F18" s="89"/>
       <c r="G18" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="H18" s="97" t="s">
+      <c r="H18" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="97"/>
-      <c r="J18" s="43" t="s">
+      <c r="I18" s="33"/>
+      <c r="J18" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="K18" s="43"/>
-      <c r="L18" s="84" t="s">
+      <c r="K18" s="89"/>
+      <c r="L18" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="M18" s="84"/>
-      <c r="N18" s="30" t="s">
+      <c r="M18" s="82"/>
+      <c r="N18" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="O18" s="31"/>
+      <c r="O18" s="28"/>
       <c r="P18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q18" s="26" t="s">
+      <c r="Q18" s="93" t="s">
         <v>30</v>
       </c>
-      <c r="R18" s="26"/>
+      <c r="R18" s="93"/>
     </row>
     <row r="19" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="42"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="43"/>
+      <c r="B19" s="88"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="89"/>
+      <c r="E19" s="89"/>
+      <c r="F19" s="89"/>
       <c r="G19" s="8"/>
-      <c r="H19" s="97"/>
-      <c r="I19" s="97"/>
-      <c r="J19" s="43"/>
-      <c r="K19" s="43"/>
-      <c r="L19" s="84"/>
-      <c r="M19" s="84"/>
-      <c r="N19" s="30"/>
-      <c r="O19" s="31"/>
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="89"/>
+      <c r="L19" s="82"/>
+      <c r="M19" s="82"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="28"/>
       <c r="P19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q19" s="26"/>
-      <c r="R19" s="26"/>
+      <c r="Q19" s="93"/>
+      <c r="R19" s="93"/>
     </row>
     <row r="20" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="42"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="43"/>
+      <c r="B20" s="88"/>
+      <c r="C20" s="89"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="89"/>
       <c r="G20" s="8"/>
-      <c r="H20" s="97"/>
-      <c r="I20" s="97"/>
-      <c r="J20" s="43"/>
-      <c r="K20" s="43"/>
-      <c r="L20" s="84"/>
-      <c r="M20" s="84"/>
-      <c r="N20" s="30"/>
-      <c r="O20" s="31"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="89"/>
+      <c r="L20" s="82"/>
+      <c r="M20" s="82"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="28"/>
       <c r="P20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="26"/>
+      <c r="Q20" s="93"/>
+      <c r="R20" s="93"/>
     </row>
     <row r="21" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="42"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
+      <c r="B21" s="88"/>
+      <c r="C21" s="89"/>
+      <c r="D21" s="89"/>
+      <c r="E21" s="89"/>
+      <c r="F21" s="89"/>
       <c r="G21" s="8"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="43"/>
-      <c r="K21" s="43"/>
-      <c r="L21" s="84"/>
-      <c r="M21" s="84"/>
-      <c r="N21" s="30"/>
-      <c r="O21" s="31"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="89"/>
+      <c r="K21" s="89"/>
+      <c r="L21" s="82"/>
+      <c r="M21" s="82"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="28"/>
       <c r="P21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q21" s="26"/>
-      <c r="R21" s="26"/>
+      <c r="Q21" s="93"/>
+      <c r="R21" s="93"/>
     </row>
     <row r="22" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="42"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
+      <c r="B22" s="88"/>
+      <c r="C22" s="89"/>
+      <c r="D22" s="89"/>
+      <c r="E22" s="89"/>
+      <c r="F22" s="89"/>
       <c r="G22" s="8"/>
-      <c r="H22" s="97"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="43"/>
-      <c r="K22" s="43"/>
-      <c r="L22" s="84"/>
-      <c r="M22" s="84"/>
-      <c r="N22" s="30"/>
-      <c r="O22" s="31"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="89"/>
+      <c r="K22" s="89"/>
+      <c r="L22" s="82"/>
+      <c r="M22" s="82"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="28"/>
       <c r="P22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q22" s="26"/>
-      <c r="R22" s="26"/>
+      <c r="Q22" s="93"/>
+      <c r="R22" s="93"/>
     </row>
     <row r="23" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="42"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
+      <c r="B23" s="88"/>
+      <c r="C23" s="89"/>
+      <c r="D23" s="89"/>
+      <c r="E23" s="89"/>
+      <c r="F23" s="89"/>
       <c r="G23" s="8"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="43"/>
-      <c r="K23" s="43"/>
-      <c r="L23" s="84"/>
-      <c r="M23" s="84"/>
-      <c r="N23" s="30"/>
-      <c r="O23" s="31"/>
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="89"/>
+      <c r="L23" s="82"/>
+      <c r="M23" s="82"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="28"/>
       <c r="P23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q23" s="26"/>
-      <c r="R23" s="26"/>
+      <c r="Q23" s="93"/>
+      <c r="R23" s="93"/>
     </row>
     <row r="24" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="42"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
+      <c r="B24" s="88"/>
+      <c r="C24" s="89"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="89"/>
+      <c r="F24" s="89"/>
       <c r="G24" s="8"/>
-      <c r="H24" s="97"/>
-      <c r="I24" s="97"/>
-      <c r="J24" s="43"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="84"/>
-      <c r="M24" s="84"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="31"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="89"/>
+      <c r="K24" s="89"/>
+      <c r="L24" s="82"/>
+      <c r="M24" s="82"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="28"/>
       <c r="P24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q24" s="26"/>
-      <c r="R24" s="26"/>
+      <c r="Q24" s="93"/>
+      <c r="R24" s="93"/>
     </row>
     <row r="25" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="42"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
+      <c r="B25" s="88"/>
+      <c r="C25" s="89"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="89"/>
+      <c r="F25" s="89"/>
       <c r="G25" s="8"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="43"/>
-      <c r="K25" s="43"/>
-      <c r="L25" s="84"/>
-      <c r="M25" s="84"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="31"/>
+      <c r="H25" s="33"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="89"/>
+      <c r="K25" s="89"/>
+      <c r="L25" s="82"/>
+      <c r="M25" s="82"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="28"/>
       <c r="P25" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q25" s="26"/>
-      <c r="R25" s="26"/>
+      <c r="Q25" s="93"/>
+      <c r="R25" s="93"/>
     </row>
     <row r="26" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="42"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="89"/>
+      <c r="D26" s="89"/>
+      <c r="E26" s="89"/>
+      <c r="F26" s="89"/>
       <c r="G26" s="8"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="43"/>
-      <c r="L26" s="84"/>
-      <c r="M26" s="84"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="31"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="33"/>
+      <c r="J26" s="89"/>
+      <c r="K26" s="89"/>
+      <c r="L26" s="82"/>
+      <c r="M26" s="82"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="28"/>
       <c r="P26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q26" s="26"/>
-      <c r="R26" s="26"/>
+      <c r="Q26" s="93"/>
+      <c r="R26" s="93"/>
     </row>
     <row r="27" spans="2:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="42"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
+      <c r="B27" s="88"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="89"/>
+      <c r="F27" s="89"/>
       <c r="G27" s="8"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="84"/>
-      <c r="M27" s="84"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="31"/>
+      <c r="H27" s="33"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="89"/>
+      <c r="K27" s="89"/>
+      <c r="L27" s="82"/>
+      <c r="M27" s="82"/>
+      <c r="N27" s="27"/>
+      <c r="O27" s="28"/>
       <c r="P27" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q27" s="26"/>
-      <c r="R27" s="26"/>
+      <c r="Q27" s="93"/>
+      <c r="R27" s="93"/>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B28" s="95" t="s">
+      <c r="B28" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="95"/>
-      <c r="D28" s="95"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="95"/>
-      <c r="I28" s="95"/>
-      <c r="J28" s="95"/>
-      <c r="K28" s="95"/>
-      <c r="L28" s="95"/>
-      <c r="M28" s="95"/>
-      <c r="N28" s="92" t="s">
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+      <c r="K28" s="47"/>
+      <c r="L28" s="47"/>
+      <c r="M28" s="47"/>
+      <c r="N28" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="O28" s="93"/>
-      <c r="P28" s="93"/>
-      <c r="Q28" s="93"/>
+      <c r="O28" s="31"/>
+      <c r="P28" s="31"/>
+      <c r="Q28" s="31"/>
       <c r="R28" s="2" t="s">
         <v>9</v>
       </c>
@@ -1686,10 +1689,10 @@
       <c r="R29" s="21"/>
     </row>
     <row r="30" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B30" s="94" t="s">
+      <c r="B30" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="C30" s="54"/>
+      <c r="C30" s="46"/>
       <c r="R30" s="22"/>
     </row>
     <row r="31" spans="2:18" x14ac:dyDescent="0.25">
@@ -1698,29 +1701,29 @@
         <v>33</v>
       </c>
       <c r="E31" s="14"/>
-      <c r="F31" s="50" t="s">
+      <c r="F31" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="G31" s="54" t="s">
+      <c r="G31" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="H31" s="54"/>
-      <c r="I31" s="48" t="s">
+      <c r="H31" s="46"/>
+      <c r="I31" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="J31" s="49">
+      <c r="J31" s="86">
         <v>1</v>
       </c>
-      <c r="K31" s="49"/>
-      <c r="L31" s="49"/>
-      <c r="M31" s="49"/>
-      <c r="N31" s="51" t="s">
+      <c r="K31" s="86"/>
+      <c r="L31" s="86"/>
+      <c r="M31" s="86"/>
+      <c r="N31" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="O31" s="49" t="s">
+      <c r="O31" s="86" t="s">
         <v>37</v>
       </c>
-      <c r="P31" s="48" t="s">
+      <c r="P31" s="62" t="s">
         <v>39</v>
       </c>
       <c r="R31" s="22"/>
@@ -1731,19 +1734,19 @@
         <v>40</v>
       </c>
       <c r="E32" s="14"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="54" t="s">
+      <c r="F32" s="29"/>
+      <c r="G32" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="H32" s="54"/>
-      <c r="I32" s="48"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="49"/>
-      <c r="L32" s="49"/>
-      <c r="M32" s="49"/>
-      <c r="N32" s="51"/>
-      <c r="O32" s="49"/>
-      <c r="P32" s="48"/>
+      <c r="H32" s="46"/>
+      <c r="I32" s="62"/>
+      <c r="J32" s="86"/>
+      <c r="K32" s="86"/>
+      <c r="L32" s="86"/>
+      <c r="M32" s="86"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="86"/>
+      <c r="P32" s="62"/>
       <c r="R32" s="22"/>
     </row>
     <row r="33" spans="2:18" x14ac:dyDescent="0.25">
@@ -1752,61 +1755,61 @@
       <c r="R33" s="23"/>
     </row>
     <row r="34" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B34" s="32" t="s">
+      <c r="B34" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="32"/>
-      <c r="I34" s="32"/>
-      <c r="J34" s="32"/>
-      <c r="K34" s="32"/>
-      <c r="L34" s="32"/>
-      <c r="M34" s="32"/>
-      <c r="N34" s="32"/>
-      <c r="O34" s="32"/>
-      <c r="P34" s="32"/>
-      <c r="Q34" s="32"/>
-      <c r="R34" s="32"/>
+      <c r="C34" s="66"/>
+      <c r="D34" s="66"/>
+      <c r="E34" s="66"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="66"/>
+      <c r="H34" s="66"/>
+      <c r="I34" s="66"/>
+      <c r="J34" s="66"/>
+      <c r="K34" s="66"/>
+      <c r="L34" s="66"/>
+      <c r="M34" s="66"/>
+      <c r="N34" s="66"/>
+      <c r="O34" s="66"/>
+      <c r="P34" s="66"/>
+      <c r="Q34" s="66"/>
+      <c r="R34" s="66"/>
     </row>
     <row r="35" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B35" s="56" t="s">
+      <c r="B35" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="57"/>
-      <c r="D35" s="57"/>
-      <c r="E35" s="57"/>
-      <c r="F35" s="57"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="59" t="s">
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="44"/>
+      <c r="H35" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="I35" s="60"/>
-      <c r="J35" s="56" t="s">
+      <c r="I35" s="61"/>
+      <c r="J35" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="K35" s="58"/>
-      <c r="L35" s="56" t="s">
+      <c r="K35" s="44"/>
+      <c r="L35" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="M35" s="57"/>
-      <c r="N35" s="57"/>
-      <c r="O35" s="58"/>
-      <c r="P35" s="55" t="s">
+      <c r="M35" s="43"/>
+      <c r="N35" s="43"/>
+      <c r="O35" s="44"/>
+      <c r="P35" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="Q35" s="55"/>
-      <c r="R35" s="55"/>
+      <c r="Q35" s="59"/>
+      <c r="R35" s="59"/>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B36" s="92" t="s">
+      <c r="B36" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="93"/>
-      <c r="D36" s="93"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
       <c r="E36" s="11" t="s">
         <v>50</v>
       </c>
@@ -1819,149 +1822,261 @@
       <c r="H36" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="I36" s="107" t="s">
+      <c r="I36" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J36" s="31" t="s">
+      <c r="J36" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="K36" s="96"/>
-      <c r="L36" s="30"/>
-      <c r="M36" s="31"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="96"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="96"/>
+      <c r="K36" s="32"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="28"/>
+      <c r="N36" s="28"/>
+      <c r="O36" s="32"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="28"/>
+      <c r="R36" s="32"/>
     </row>
     <row r="37" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="46"/>
-      <c r="C37" s="88"/>
-      <c r="D37" s="88"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
       <c r="E37" s="9"/>
       <c r="F37" s="24"/>
       <c r="G37" s="9"/>
       <c r="H37" s="25"/>
-      <c r="I37" s="107" t="s">
+      <c r="I37" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J37" s="31"/>
-      <c r="K37" s="96"/>
-      <c r="L37" s="30"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="96"/>
-      <c r="P37" s="30"/>
-      <c r="Q37" s="31"/>
-      <c r="R37" s="96"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="32"/>
+      <c r="L37" s="27"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="28"/>
+      <c r="O37" s="32"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="32"/>
     </row>
     <row r="38" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="46"/>
-      <c r="C38" s="88"/>
-      <c r="D38" s="88"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="35"/>
       <c r="E38" s="9"/>
       <c r="F38" s="24"/>
       <c r="G38" s="9"/>
       <c r="H38" s="25"/>
-      <c r="I38" s="107" t="s">
+      <c r="I38" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J38" s="31"/>
-      <c r="K38" s="96"/>
-      <c r="L38" s="30"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-      <c r="O38" s="96"/>
-      <c r="P38" s="30"/>
-      <c r="Q38" s="31"/>
-      <c r="R38" s="96"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="32"/>
+      <c r="L38" s="27"/>
+      <c r="M38" s="28"/>
+      <c r="N38" s="28"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="27"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="32"/>
     </row>
     <row r="39" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="46"/>
-      <c r="C39" s="88"/>
-      <c r="D39" s="88"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="35"/>
+      <c r="D39" s="35"/>
       <c r="E39" s="9"/>
       <c r="F39" s="24"/>
       <c r="G39" s="9"/>
       <c r="H39" s="25"/>
-      <c r="I39" s="107" t="s">
+      <c r="I39" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J39" s="31"/>
-      <c r="K39" s="96"/>
-      <c r="L39" s="30"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
-      <c r="O39" s="96"/>
-      <c r="P39" s="30"/>
-      <c r="Q39" s="31"/>
-      <c r="R39" s="96"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="32"/>
+      <c r="L39" s="27"/>
+      <c r="M39" s="28"/>
+      <c r="N39" s="28"/>
+      <c r="O39" s="32"/>
+      <c r="P39" s="27"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="32"/>
     </row>
     <row r="40" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="46"/>
-      <c r="C40" s="88"/>
-      <c r="D40" s="88"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
       <c r="E40" s="9"/>
       <c r="F40" s="24"/>
       <c r="G40" s="9"/>
       <c r="H40" s="25"/>
-      <c r="I40" s="107" t="s">
+      <c r="I40" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J40" s="31"/>
-      <c r="K40" s="96"/>
-      <c r="L40" s="30"/>
-      <c r="M40" s="31"/>
-      <c r="N40" s="31"/>
-      <c r="O40" s="96"/>
-      <c r="P40" s="30"/>
-      <c r="Q40" s="31"/>
-      <c r="R40" s="96"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="32"/>
+      <c r="L40" s="27"/>
+      <c r="M40" s="28"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="32"/>
+      <c r="P40" s="27"/>
+      <c r="Q40" s="28"/>
+      <c r="R40" s="32"/>
     </row>
     <row r="41" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="46"/>
-      <c r="C41" s="88"/>
-      <c r="D41" s="88"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
       <c r="E41" s="9"/>
       <c r="F41" s="24"/>
       <c r="G41" s="9"/>
       <c r="H41" s="25"/>
-      <c r="I41" s="107" t="s">
+      <c r="I41" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J41" s="31"/>
-      <c r="K41" s="96"/>
-      <c r="L41" s="30"/>
-      <c r="M41" s="31"/>
-      <c r="N41" s="31"/>
-      <c r="O41" s="96"/>
-      <c r="P41" s="30"/>
-      <c r="Q41" s="31"/>
-      <c r="R41" s="96"/>
+      <c r="J41" s="28"/>
+      <c r="K41" s="32"/>
+      <c r="L41" s="27"/>
+      <c r="M41" s="28"/>
+      <c r="N41" s="28"/>
+      <c r="O41" s="32"/>
+      <c r="P41" s="27"/>
+      <c r="Q41" s="28"/>
+      <c r="R41" s="32"/>
     </row>
     <row r="42" spans="2:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="46"/>
-      <c r="C42" s="88"/>
-      <c r="D42" s="88"/>
+      <c r="B42" s="34"/>
+      <c r="C42" s="35"/>
+      <c r="D42" s="35"/>
       <c r="E42" s="9"/>
       <c r="F42" s="24"/>
       <c r="G42" s="9"/>
       <c r="H42" s="25"/>
-      <c r="I42" s="107" t="s">
+      <c r="I42" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J42" s="31"/>
-      <c r="K42" s="96"/>
-      <c r="L42" s="30"/>
-      <c r="M42" s="31"/>
-      <c r="N42" s="31"/>
-      <c r="O42" s="96"/>
-      <c r="P42" s="30"/>
-      <c r="Q42" s="31"/>
-      <c r="R42" s="96"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="32"/>
+      <c r="L42" s="27"/>
+      <c r="M42" s="28"/>
+      <c r="N42" s="28"/>
+      <c r="O42" s="32"/>
+      <c r="P42" s="27"/>
+      <c r="Q42" s="28"/>
+      <c r="R42" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="136">
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="B2:R2"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="B16:R16"/>
+    <mergeCell ref="B12:R12"/>
+    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="B15:P15"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B6:C7"/>
+    <mergeCell ref="B8:C9"/>
+    <mergeCell ref="B10:C11"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="Q26:R26"/>
+    <mergeCell ref="Q27:R27"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="I7:L11"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:M32"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="L42:O42"/>
+    <mergeCell ref="L36:O36"/>
+    <mergeCell ref="L37:O37"/>
+    <mergeCell ref="P35:R35"/>
+    <mergeCell ref="L35:O35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="B17:K17"/>
+    <mergeCell ref="B34:R34"/>
+    <mergeCell ref="M6:O6"/>
+    <mergeCell ref="M7:O11"/>
+    <mergeCell ref="P6:R6"/>
+    <mergeCell ref="P7:R11"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="D8:E9"/>
+    <mergeCell ref="D10:E11"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B28:M28"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F7:H8"/>
+    <mergeCell ref="F10:H11"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="L38:O38"/>
+    <mergeCell ref="L39:O39"/>
+    <mergeCell ref="L40:O40"/>
+    <mergeCell ref="L41:O41"/>
     <mergeCell ref="N23:O23"/>
     <mergeCell ref="N31:N32"/>
     <mergeCell ref="N28:Q28"/>
@@ -1986,118 +2101,6 @@
     <mergeCell ref="P40:R40"/>
     <mergeCell ref="J38:K38"/>
     <mergeCell ref="J39:K39"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="D6:E7"/>
-    <mergeCell ref="D8:E9"/>
-    <mergeCell ref="D10:E11"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B28:M28"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F7:H8"/>
-    <mergeCell ref="F10:H11"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="L38:O38"/>
-    <mergeCell ref="L39:O39"/>
-    <mergeCell ref="L40:O40"/>
-    <mergeCell ref="L41:O41"/>
-    <mergeCell ref="L42:O42"/>
-    <mergeCell ref="L36:O36"/>
-    <mergeCell ref="L37:O37"/>
-    <mergeCell ref="P35:R35"/>
-    <mergeCell ref="L35:O35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="B17:K17"/>
-    <mergeCell ref="B34:R34"/>
-    <mergeCell ref="M6:O6"/>
-    <mergeCell ref="M7:O11"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="P7:R11"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="I7:L11"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="P31:P32"/>
-    <mergeCell ref="O31:O32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="J31:M32"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B14:I14"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="Q26:R26"/>
-    <mergeCell ref="Q27:R27"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="J14:M14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="B16:R16"/>
-    <mergeCell ref="B12:R12"/>
-    <mergeCell ref="B13:P13"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="B15:P15"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B6:C7"/>
-    <mergeCell ref="B8:C9"/>
-    <mergeCell ref="B10:C11"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
   </mergeCells>
   <pageMargins left="0.1" right="0.1" top="0.2" bottom="0.75" header="0.1" footer="0.3"/>
   <pageSetup scale="71" orientation="portrait" r:id="rId1"/>
@@ -2105,18 +2108,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2246,6 +2249,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14EA48F8-1535-4600-B361-5A56BC1EA18D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="b7409cf6-e852-4a78-b0e6-5ba582a53027"/>
@@ -2257,14 +2268,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A727A15-14BD-4411-9BCA-DFC33A70ED4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>